<commit_message>
add CJM select function
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_limit_torque_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_limit_torque_calc.xlsx
@@ -480,22 +480,22 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>13.47774891631924</v>
+        <v>10.20241688096769</v>
       </c>
       <c r="B2" t="n">
-        <v>-72.00936976614922</v>
+        <v>-51.08155090132491</v>
       </c>
       <c r="C2" t="n">
-        <v>-34.25216425596847</v>
+        <v>-22.7933814227316</v>
       </c>
       <c r="D2" t="n">
-        <v>-2.811438983146238</v>
+        <v>-1.740564174316093</v>
       </c>
       <c r="E2" t="n">
-        <v>0.09277585571694945</v>
+        <v>0.05619287391438826</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0004908700000088073</v>
+        <v>0.0004908700000088069</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -510,27 +510,27 @@
         <v>180</v>
       </c>
       <c r="K2" t="n">
-        <v>-90</v>
+        <v>90</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>-180</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-7.772383609049233</v>
+        <v>-5.290733031250725</v>
       </c>
       <c r="B3" t="n">
-        <v>50.36154278639225</v>
+        <v>38.6883258584235</v>
       </c>
       <c r="C3" t="n">
-        <v>11.47090011521701</v>
+        <v>9.047703354877688</v>
       </c>
       <c r="D3" t="n">
-        <v>2.122940732096838</v>
+        <v>1.28285349628316</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.1165421032237456</v>
+        <v>-0.0701672651549502</v>
       </c>
       <c r="F3" t="n">
         <v>0.0004908700000088066</v>
@@ -556,19 +556,19 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>6.972533808792097</v>
+        <v>5.938985313002886</v>
       </c>
       <c r="B4" t="n">
-        <v>107.2308603668059</v>
+        <v>75.98181890618442</v>
       </c>
       <c r="C4" t="n">
-        <v>54.42167729600679</v>
+        <v>36.19331783428503</v>
       </c>
       <c r="D4" t="n">
-        <v>9.180845729239461</v>
+        <v>5.26335277486748</v>
       </c>
       <c r="E4" t="n">
-        <v>0.07414737338717628</v>
+        <v>0.04488511875415421</v>
       </c>
       <c r="F4" t="n">
         <v>0.002454350000002935</v>
@@ -577,7 +577,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>-180</v>
+        <v>180</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -594,19 +594,19 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>11.22292532591712</v>
+        <v>8.712861580632017</v>
       </c>
       <c r="B5" t="n">
-        <v>-80.64165378982474</v>
+        <v>-56.06433124095879</v>
       </c>
       <c r="C5" t="n">
-        <v>-40.5206617459604</v>
+        <v>-26.27610193289824</v>
       </c>
       <c r="D5" t="n">
-        <v>-6.716149939454543</v>
+        <v>-3.723224855015485</v>
       </c>
       <c r="E5" t="n">
-        <v>0.05421614203604733</v>
+        <v>0.03384697848175559</v>
       </c>
       <c r="F5" t="n">
         <v>-0.0004908699999853221</v>
@@ -632,19 +632,19 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>4.912938711212601</v>
+        <v>3.802259157163413</v>
       </c>
       <c r="B6" t="n">
-        <v>42.58138142394621</v>
+        <v>26.63651949907414</v>
       </c>
       <c r="C6" t="n">
-        <v>54.71371440060757</v>
+        <v>36.51337799168403</v>
       </c>
       <c r="D6" t="n">
-        <v>9.266341622255835</v>
+        <v>5.316335649682959</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1026285514034496</v>
+        <v>0.06252644241314888</v>
       </c>
       <c r="F6" t="n">
         <v>0.002454350000002935</v>
@@ -670,19 +670,19 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1.038274895355398</v>
+        <v>0.5612445370203584</v>
       </c>
       <c r="B7" t="n">
-        <v>-34.00100282035061</v>
+        <v>-22.81515460382354</v>
       </c>
       <c r="C7" t="n">
-        <v>-44.34289242548079</v>
+        <v>-29.06319697823687</v>
       </c>
       <c r="D7" t="n">
-        <v>-7.409164794611282</v>
+        <v>-4.164466565455585</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.0312622979940821</v>
+        <v>-0.01911626172420416</v>
       </c>
       <c r="F7" t="n">
         <v>-0.0004908699999853231</v>
@@ -708,19 +708,19 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2.233718475185733</v>
+        <v>1.23089958172399</v>
       </c>
       <c r="B8" t="n">
-        <v>9.715152813900735</v>
+        <v>4.811234318230071</v>
       </c>
       <c r="C8" t="n">
-        <v>10.44772444685643</v>
+        <v>5.898938693097441</v>
       </c>
       <c r="D8" t="n">
-        <v>10.13038316942368</v>
+        <v>5.863582378979679</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1880371794709396</v>
+        <v>0.1154111441611366</v>
       </c>
       <c r="F8" t="n">
         <v>0.002454350000002935</v>
@@ -746,19 +746,19 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>-0.4536655114448799</v>
+        <v>-0.5757737499049899</v>
       </c>
       <c r="B9" t="n">
-        <v>2.862344280065093</v>
+        <v>1.607468904054138</v>
       </c>
       <c r="C9" t="n">
-        <v>-2.879394166354958</v>
+        <v>-1.434825570012902</v>
       </c>
       <c r="D9" t="n">
-        <v>-9.671045523163453</v>
+        <v>-5.600180733065074</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1661661157091655</v>
+        <v>0.1023938979680933</v>
       </c>
       <c r="F9" t="n">
         <v>0.001472609999985322</v>
@@ -784,19 +784,19 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2.098794470644656</v>
+        <v>1.149952597581742</v>
       </c>
       <c r="B10" t="n">
-        <v>9.173383996798824</v>
+        <v>4.475683099361846</v>
       </c>
       <c r="C10" t="n">
-        <v>10.1339097718287</v>
+        <v>5.704635871188161</v>
       </c>
       <c r="D10" t="n">
-        <v>10.04452263647013</v>
+        <v>5.810527954029345</v>
       </c>
       <c r="E10" t="n">
-        <v>0.8641756390893633</v>
+        <v>0.4871734209400908</v>
       </c>
       <c r="F10" t="n">
         <v>0.001472609999979452</v>
@@ -822,19 +822,19 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2.271418918734376</v>
+        <v>1.257153919485134</v>
       </c>
       <c r="B11" t="n">
-        <v>9.956871465341285</v>
+        <v>4.961392830305935</v>
       </c>
       <c r="C11" t="n">
-        <v>10.51869565412466</v>
+        <v>5.943406340135321</v>
       </c>
       <c r="D11" t="n">
-        <v>10.03060693251959</v>
+        <v>5.802359160979575</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.8573084985497497</v>
+        <v>-0.4808182805149171</v>
       </c>
       <c r="F11" t="n">
         <v>-0.0004908700000205485</v>
@@ -852,27 +852,27 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
+        <v>180</v>
+      </c>
+      <c r="L11" t="n">
         <v>-180</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>5.736607171775577</v>
+        <v>5.246506406687828</v>
       </c>
       <c r="B12" t="n">
-        <v>-79.14258238567194</v>
+        <v>-55.64134205681706</v>
       </c>
       <c r="C12" t="n">
-        <v>-35.40452142225948</v>
+        <v>-23.54071019335533</v>
       </c>
       <c r="D12" t="n">
-        <v>2.017059303794476</v>
+        <v>1.324569439928595</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.01362087101736764</v>
+        <v>-0.0121404359254656</v>
       </c>
       <c r="F12" t="n">
         <v>0.003436090000008806</v>
@@ -898,19 +898,19 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>5.593003761241677</v>
+        <v>5.158135872179554</v>
       </c>
       <c r="B13" t="n">
-        <v>-78.25866068004262</v>
+        <v>-55.19019540189476</v>
       </c>
       <c r="C13" t="n">
-        <v>-34.34950321264454</v>
+        <v>-22.98347998110509</v>
       </c>
       <c r="D13" t="n">
-        <v>3.243174017395036</v>
+        <v>1.987883209506788</v>
       </c>
       <c r="E13" t="n">
-        <v>0.01367252879253835</v>
+        <v>0.0121920937006363</v>
       </c>
       <c r="F13" t="n">
         <v>-0.002454350000008806</v>
@@ -968,19 +968,19 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>13.47774891631924</v>
+        <v>10.20241688096769</v>
       </c>
       <c r="B15" t="n">
-        <v>107.2308603668059</v>
+        <v>75.98181890618442</v>
       </c>
       <c r="C15" t="n">
-        <v>54.71371440060757</v>
+        <v>36.51337799168403</v>
       </c>
       <c r="D15" t="n">
-        <v>10.13038316942368</v>
+        <v>5.863582378979679</v>
       </c>
       <c r="E15" t="n">
-        <v>0.8641756390893633</v>
+        <v>0.4871734209400908</v>
       </c>
       <c r="F15" t="n">
         <v>0.003436090000008806</v>

</xml_diff>

<commit_message>
TODO: fix stl conv 6dof urdf & 修改為可調整dof的方式
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_limit_torque_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_limit_torque_calc.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col customWidth="1" max="1" min="1" width="20"/>
@@ -439,8 +439,6 @@
     <col customWidth="1" max="10" min="10" width="20"/>
     <col customWidth="1" max="11" min="11" width="20"/>
     <col customWidth="1" max="12" min="12" width="20"/>
-    <col customWidth="1" max="13" min="13" width="20"/>
-    <col customWidth="1" max="14" min="14" width="20"/>
   </cols>
   <sheetData>
     <row customHeight="1" ht="40" r="1">
@@ -476,63 +474,53 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>torque 7</t>
+          <t>angle 1</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>angle 1</t>
+          <t>angle 2</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>angle 2</t>
+          <t>angle 3</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>angle 3</t>
+          <t>angle 4</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>angle 4</t>
+          <t>angle 5</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>angle 5</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
           <t>angle 6</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>angle 7</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>3.944304526105059e-31</v>
+        <v>22.60661927447309</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>-8.41364346382081</v>
+        <v>-22.59356694474243</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.1635899709951098</v>
+        <v>-14.06881746673712</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2.515714543312775</v>
+        <v>-6.051374667215467</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.0007568300337062456</v>
+        <v>0.1655815129150472</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-3.79405811189483e-17</v>
+        <v>0.001156584958283194</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0</v>
@@ -541,130 +529,112 @@
         <v>0</v>
       </c>
       <c r="I2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="K2" s="2" t="n">
         <v>-90</v>
       </c>
-      <c r="J2" s="2" t="n">
-        <v>-180</v>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="L2" s="2" t="n">
-        <v>-90</v>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>-180</v>
-      </c>
-      <c r="N2" s="2" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>-5.916456789157589e-31</v>
+        <v>-18.45100483697522</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>8.41364346382081</v>
+        <v>30.32353446810498</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>-0.1635899709951098</v>
+        <v>21.63598421662745</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>-2.515714543312775</v>
+        <v>1.701200208414609</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-0.0007568300337062568</v>
+        <v>0.2836898492433492</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-1.897029197763442e-17</v>
+        <v>-0.008175415684367393</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>90</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>180</v>
+        <v>-180</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L3" s="2" t="n">
         <v>-90</v>
       </c>
-      <c r="M3" s="2" t="n">
-        <v>180</v>
-      </c>
-      <c r="N3" s="2" t="n">
-        <v>90</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>-1.97215226305253e-31</v>
+        <v>12.96406004405746</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>8.72345184270756</v>
+        <v>57.32907156079247</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.2356216378120972</v>
+        <v>28.00104595853756</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2.825522922199525</v>
+        <v>-5.470927493063819</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.07278849685069361</v>
+        <v>-0.4562877668026663</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.1549041894433748</v>
+        <v>0.004626339833147555</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0</v>
+        <v>-180</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0</v>
+        <v>-180</v>
       </c>
       <c r="K4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="2" t="n">
-        <v>90</v>
+        <v>-180</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>0</v>
+        <v>3.34028712355232</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>-8.72345184270756</v>
+        <v>-39.42535058705666</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.2356216378120972</v>
+        <v>-18.74577924073374</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>-2.825522922199525</v>
+        <v>6.288414174432563</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>-0.07278849685069361</v>
+        <v>0.5229734554954202</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-0.1549041894433748</v>
+        <v>0.004626339832951993</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>0</v>
@@ -673,7 +643,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>-90</v>
+        <v>0</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>0</v>
@@ -682,39 +652,33 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="2" t="n">
         <v>90</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>0</v>
+        <v>5.183317671921121</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>6.357852002062653</v>
+        <v>14.17102947076536</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3.442918480467286</v>
+        <v>34.88092866295083</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>3.460267602589124e-16</v>
+        <v>6.002614967706206</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.0007567837130766367</v>
+        <v>0.182295454986041</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1.897029197763442e-17</v>
+        <v>0.01048858560098513</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>90</v>
@@ -723,86 +687,74 @@
         <v>-90</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>90</v>
+        <v>-90</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="2" t="n">
         <v>90</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>4.930380657631324e-32</v>
+        <v>-4.104398608859751</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>6.357852002062653</v>
+        <v>-8.20753999592924</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-3.442918480467286</v>
+        <v>-23.58822497645226</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>5.632433296798498e-17</v>
+        <v>5.258950143876911</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-0.0007567837130766278</v>
+        <v>0.4373921972986484</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>2.836320541018949e-24</v>
+        <v>0.004626339832951993</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>90</v>
+        <v>-90</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="2" t="n">
         <v>90</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>2.465190328815662e-32</v>
+        <v>3.107484036648333</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>3.439704723237628</v>
+        <v>1.267263831394952</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>4.21635909682953e-16</v>
+        <v>4.146154727500027</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>2.825522922199525</v>
+        <v>9.330657670349888</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.07278849685069361</v>
+        <v>0.4543963148261407</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>0.1549041894433748</v>
+        <v>0.01048858560098513</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="I8" s="2" t="n">
         <v>0</v>
@@ -811,168 +763,144 @@
         <v>0</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>90</v>
+        <v>-90</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="2" t="n">
         <v>90</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>9.860761315262648e-32</v>
+        <v>-2.647647570629449</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>-2.211341121161422</v>
+        <v>14.25217672214665</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-2.704176108348719e-16</v>
+        <v>4.205002015290807</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>-2.825522922199525</v>
+        <v>-8.706986886004621</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-0.07278849685069361</v>
+        <v>0.4005060688280094</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>-0.1549041894433748</v>
+        <v>0.008175415684418742</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="I9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0</v>
+        <v>-180</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>-90</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="2" t="n">
-        <v>90</v>
+        <v>-180</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>1.725633230170963e-31</v>
+        <v>2.933329164887276</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>-3.291228071413882</v>
+        <v>0.4339840543235947</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-4.026656205416392e-16</v>
+        <v>3.623318767900233</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>2.670618755916465</v>
+        <v>9.242443055210282</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.1556609963167663</v>
+        <v>0.7864416251388029</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>1.89702976502755e-17</v>
+        <v>0.001901201271454379</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="I10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>-90</v>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="N10" s="2" t="n">
         <v>90</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>1.479114197289397e-31</v>
+        <v>3.070971564483818</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>6.514269782092496</v>
+        <v>2.092889319742423</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>3.288014314184225</v>
+        <v>4.58302808270107</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>3.270564711175985e-16</v>
+        <v>9.223278039145931</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-0.1556609963167663</v>
+        <v>-0.7572814126529369</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>-1.89702976502755e-17</v>
+        <v>0.0004119686448611116</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>-90</v>
+        <v>0</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
       <c r="L11" s="2" t="n">
         <v>-180</v>
       </c>
-      <c r="M11" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="N11" s="2" t="n">
-        <v>90</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>3.081487911019577e-33</v>
+        <v>3.967498803901822</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.3091629320871749</v>
+        <v>-38.77125130577514</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>3.82551112700106e-17</v>
+        <v>-18.48770503512054</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>-0.3050188689509281</v>
+        <v>5.99205327411009</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1.906297408914157e-17</v>
+        <v>0.07332223507582536</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.1549041894433748</v>
+        <v>0.01750741632722737</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>0</v>
@@ -987,36 +915,30 @@
         <v>0</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>0</v>
+        <v>-90</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="N12" s="2" t="n">
         <v>90</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>-7.113903732080352e-33</v>
+        <v>3.758339881912064</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>-0.0006454467995747181</v>
+        <v>-38.51186721564472</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3.145273147417692e-19</v>
+        <v>-18.08903964391211</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>-0.6148272478376777</v>
+        <v>6.585712486827747</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-1.887760986612726e-17</v>
+        <v>-0.07303544917504008</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-0.1549041894433748</v>
+        <v>-0.01519424641070249</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>0</v>
@@ -1031,179 +953,75 @@
         <v>0</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>-90</v>
-      </c>
-      <c r="N13" s="2" t="n">
         <v>90</v>
       </c>
     </row>
     <row customHeight="1" ht="40" r="14">
-      <c r="A14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="1" t="n">
-        <v>0</v>
-      </c>
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Torque 1 max</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>Torque 2 max</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>Torque 3 max</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Torque 4 max</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Torque 5 max</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>Torque 6 max</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="n"/>
+      <c r="H14" s="1" t="n"/>
+      <c r="I14" s="1" t="n"/>
+      <c r="J14" s="1" t="n"/>
+      <c r="K14" s="1" t="n"/>
+      <c r="L14" s="1" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>0</v>
+        <v>22.60661927447309</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>57.32907156079247</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0</v>
+        <v>34.88092866295083</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0</v>
+        <v>9.330657670349888</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0</v>
+        <v>0.7864416251388029</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Torque 1 max</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Torque 2 max</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Torque 3 max</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Torque 4 max</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Torque 5 max</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Torque 6 max</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Torque 7 max</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="n"/>
-      <c r="K16" s="2" t="n"/>
-      <c r="L16" s="2" t="n"/>
-      <c r="M16" s="2" t="n"/>
-      <c r="N16" s="2" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>3.944304526105059e-31</v>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>8.72345184270756</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>3.442918480467286</v>
-      </c>
-      <c r="D17" s="2" t="n">
-        <v>2.825522922199525</v>
-      </c>
-      <c r="E17" s="2" t="n">
-        <v>0.1556609963167663</v>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>0.1549041894433748</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="n"/>
-      <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="n"/>
-      <c r="N17" s="2" t="n"/>
+        <v>0.01750741632722737</v>
+      </c>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="n"/>
+      <c r="K15" s="2" t="n"/>
+      <c r="L15" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>

</xml_diff>